<commit_message>
Add shift accounting: rules, journal, КПП parser and report script
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RP3efy3v6UXZ3TFiDt8HNv
</commit_message>
<xml_diff>
--- a/reports/otchet_po_smenam.xlsx
+++ b/reports/otchet_po_smenam.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,9 +28,6 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -55,7 +52,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -63,37 +60,15 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00999999"/>
-      </left>
-      <right style="thin">
-        <color rgb="00999999"/>
-      </right>
-      <top style="thin">
-        <color rgb="00999999"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00999999"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -459,20 +434,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
     <col width="36" customWidth="1" min="2" max="2"/>
     <col width="52" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Отчет по сменам — СУПЕР-ВОВИК, КПП от 07.10.2026 (расчет на 19.10.2026)</t>
+          <t>Отчет по сменам — СУПЕР-ВОВИК, kpp_2026-10-07.xlsx</t>
         </is>
       </c>
     </row>
@@ -499,7 +474,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Накопительно (оклад + допы), ₽</t>
+          <t>Накопительно, ₽</t>
         </is>
       </c>
     </row>
@@ -519,10 +494,10 @@
           <t>Прикрепление / погрузка</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="3" t="n">
         <v>5000</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="3" t="n">
         <v>155000</v>
       </c>
     </row>
@@ -542,10 +517,10 @@
           <t>Прилет в Краснодар / разгрузка</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>5000</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="3" t="n">
         <v>160000</v>
       </c>
     </row>
@@ -565,194 +540,194 @@
           <t>Загрузка костюм / грим / АХЧ</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="3" t="n">
         <v>5000</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="3" t="n">
         <v>165000</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" t="inlineStr">
         <is>
           <t>11.10</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>СМЕНА №1 ✅</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Работа по КПП</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="6" t="n">
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" t="n">
         <v>165000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>12.10</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>СМЕНА №2 ✅</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Работа по КПП</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="6" t="n">
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
         <v>165000</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>13.10</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>СМЕНА №3 ✅</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>Работа по КПП</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="6" t="n">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
         <v>165000</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" t="inlineStr">
         <is>
           <t>14.10</t>
         </is>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>ВЫХОДНОЙ</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Не подтверждено (нет работы)</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="6" t="n">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Нет работы</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
         <v>165000</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>15.10</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>СМЕНА №4 ✅</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Работа по КПП</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="6" t="n">
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
         <v>165000</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>16.10</t>
         </is>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>СМЕНА №5 ✅</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>Работа по КПП</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="6" t="n">
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
         <v>165000</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>17.10</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>СМЕНА №1-6 ✅</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Работа по КПП</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="6" t="n">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
         <v>165000</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>18.10</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>СМЕНА №7 ✅</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>Работа по КПП</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="6" t="n">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" t="n">
         <v>165000</v>
       </c>
     </row>
@@ -764,7 +739,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>ВЫХОДНОЙ (заменен на подготовку)</t>
+          <t>ВЫХОДНОЙ</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -772,583 +747,576 @@
           <t>Смена разгрузки / заклеивание пола в локации, 11:00</t>
         </is>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" s="3" t="n">
         <v>5000</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="3" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" t="inlineStr">
         <is>
           <t>20.10</t>
         </is>
       </c>
-      <c r="B16" s="5" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>СМЕНА №8 ✅</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="6" t="n">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" t="inlineStr">
         <is>
           <t>21.10</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>СМЕНА №9 ✅</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="6" t="n">
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" t="inlineStr">
         <is>
           <t>22.10</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>СМЕНА №10 ✅</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="6" t="n">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" t="inlineStr">
         <is>
           <t>23.10</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>СМЕНА №11 ✅</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="6" t="n">
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>24.10</t>
         </is>
       </c>
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>ОТСЫПНОЙ</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Не подтверждено (нет работы)</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="6" t="n">
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Нет работы</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" t="inlineStr">
         <is>
           <t>25.10</t>
         </is>
       </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>СМЕНА №12 ✅</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="6" t="n">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" t="inlineStr">
         <is>
           <t>26.10</t>
         </is>
       </c>
-      <c r="B22" s="5" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>ВЫХОДНОЙ</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Не подтверждено (нет работы)</t>
-        </is>
-      </c>
-      <c r="D22" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="6" t="n">
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Нет работы</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>27.10</t>
         </is>
       </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>ВЫХОДНОЙ</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>Не подтверждено (нет работы)</t>
-        </is>
-      </c>
-      <c r="D23" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="6" t="n">
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Нет работы</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>28.10</t>
         </is>
       </c>
-      <c r="B24" s="5" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>ПОДГОТОВКА</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Не подтверждено (нет работы)</t>
-        </is>
-      </c>
-      <c r="D24" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="6" t="n">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Нет работы</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" t="inlineStr">
         <is>
           <t>29.10</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>СМЕНА №13 ✅</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" s="6" t="n">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
+      <c r="A26" t="inlineStr">
         <is>
           <t>30.10</t>
         </is>
       </c>
-      <c r="B26" s="5" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>СМЕНА №14 ✅</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D26" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E26" s="6" t="n">
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" t="inlineStr">
         <is>
           <t>31.10</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>СМЕНА №15 ✅</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="6" t="n">
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="A28" t="inlineStr">
         <is>
           <t>01.11</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>СМЕНА №16 ✅</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E28" s="6" t="n">
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="A29" t="inlineStr">
         <is>
           <t>02.11</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>СМЕНА №17 ✅</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" s="6" t="n">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" t="inlineStr">
         <is>
           <t>03.11</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
+      <c r="B30" t="inlineStr">
         <is>
           <t>ВЫХОДНОЙ</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Не подтверждено (нет работы)</t>
-        </is>
-      </c>
-      <c r="D30" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="6" t="n">
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Нет работы</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="A31" t="inlineStr">
         <is>
           <t>04.11</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" t="inlineStr">
         <is>
           <t>СМЕНА №18 ✅</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" s="6" t="n">
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+      <c r="A32" t="inlineStr">
         <is>
           <t>05.11</t>
         </is>
       </c>
-      <c r="B32" s="5" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>СМЕНА №19 ✅</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D32" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="6" t="n">
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+      <c r="A33" t="inlineStr">
         <is>
           <t>06.11</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>СМЕНА №20 ✅</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E33" s="6" t="n">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="A34" t="inlineStr">
         <is>
           <t>07.11</t>
         </is>
       </c>
-      <c r="B34" s="5" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>СМЕНА №21 ✅</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D34" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E34" s="6" t="n">
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="A35" t="inlineStr">
         <is>
           <t>08.11</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>ВЫХОДНОЙ</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>Не подтверждено (нет работы)</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E35" s="6" t="n">
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Нет работы</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="A36" t="inlineStr">
         <is>
           <t>09.11</t>
         </is>
       </c>
-      <c r="B36" s="5" t="inlineStr">
+      <c r="B36" t="inlineStr">
         <is>
           <t>СМЕНА №22 ✅</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E36" s="6" t="n">
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="5" t="inlineStr">
+      <c r="A37" t="inlineStr">
         <is>
           <t>10.11</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>СМЕНА №23 ✅</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>Предстоит</t>
-        </is>
-      </c>
-      <c r="D37" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E37" s="6" t="n">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Смена по КПП (в окладе)</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
         <v>170000</v>
       </c>
     </row>
     <row r="38">
-      <c r="D38" s="7" t="n"/>
-      <c r="E38" s="7" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>11.11</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>режим не указан</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Нет работы</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>170000</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
         <is>
           <t>Оклад</t>
         </is>
       </c>
-      <c r="D39" s="7" t="n"/>
-      <c r="E39" s="9" t="n">
+      <c r="E40" t="n">
         <v>150000</v>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="8" t="inlineStr">
-        <is>
-          <t>Допы (5 000 ₽ × 4)</t>
-        </is>
-      </c>
-      <c r="D40" s="7" t="n"/>
-      <c r="E40" s="9">
-        <f>SUM(D4:D37)</f>
-        <v/>
-      </c>
-    </row>
     <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Допы</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
         <is>
           <t>К выплате</t>
         </is>
       </c>
-      <c r="D41" s="7" t="n"/>
-      <c r="E41" s="9">
-        <f>E39+E40</f>
-        <v/>
+      <c r="E42" t="n">
+        <v>170000</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Съёмочных смен в окладе по КПП: 23 (отработано 7: 11–18.10; впереди 16: с 20.10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="inlineStr">
-        <is>
-          <t>Допы: тех. дни вне КПП и работа в ВЫХОДНОЙ/ОТСЫПНОЙ/ПОДГОТОВКА — по 5 000 ₽.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>Допущения: 17.10 («СМЕНА №1-6») = одна смена; 19.10 = одна доплата; 11.11 — режим в КПП не указан.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Договор подписан без акта — рекомендуется подписать акт со списком смен и допов.</t>
+          <t>Смен в окладе по КПП: 23</t>
         </is>
       </c>
     </row>

</xml_diff>